<commit_message>
Day 1 pins: add question + hook columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nix2dmocL7MmA5BQMTWtPa
</commit_message>
<xml_diff>
--- a/system/daily/Sideline_Ready_Day1_15_Pins.xlsx
+++ b/system/daily/Sideline_Ready_Day1_15_Pins.xlsx
@@ -165,9 +165,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Day1" displayName="Day1" ref="A1:S16" headerRowCount="1">
-  <autoFilter ref="A1:S16"/>
-  <tableColumns count="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Day1" displayName="Day1" ref="A1:U16" headerRowCount="1">
+  <autoFilter ref="A1:U16"/>
+  <tableColumns count="21">
     <tableColumn id="1" name="#"/>
     <tableColumn id="2" name="Day"/>
     <tableColumn id="3" name="Post time (CT)"/>
@@ -177,16 +177,18 @@
     <tableColumn id="7" name="Reviews"/>
     <tableColumn id="8" name="Bought last month"/>
     <tableColumn id="9" name="Text overlay (exact search phrase)"/>
-    <tableColumn id="10" name="Pin title"/>
-    <tableColumn id="11" name="Pin description"/>
-    <tableColumn id="12" name="Alt text"/>
-    <tableColumn id="13" name="Pinterest board"/>
-    <tableColumn id="14" name="Amazon affiliate link"/>
-    <tableColumn id="15" name="Image prompt (OpenArt / Runway)"/>
-    <tableColumn id="16" name="Video plan (8-10 sec)"/>
-    <tableColumn id="17" name="Avatar line (caption or voice)"/>
-    <tableColumn id="18" name="File name"/>
-    <tableColumn id="19" name="ASIN"/>
+    <tableColumn id="10" name="The question she's asking"/>
+    <tableColumn id="11" name="Hook (answers it, on the pin under the overlay)"/>
+    <tableColumn id="12" name="Pin title"/>
+    <tableColumn id="13" name="Pin description"/>
+    <tableColumn id="14" name="Alt text"/>
+    <tableColumn id="15" name="Pinterest board"/>
+    <tableColumn id="16" name="Amazon affiliate link"/>
+    <tableColumn id="17" name="Image prompt (OpenArt / Runway)"/>
+    <tableColumn id="18" name="Video plan (8-10 sec)"/>
+    <tableColumn id="19" name="Avatar line (caption or voice)"/>
+    <tableColumn id="20" name="File name"/>
+    <tableColumn id="21" name="ASIN"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -481,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -493,16 +495,18 @@
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="55" customWidth="1" min="15" max="15"/>
-    <col width="55" customWidth="1" min="16" max="16"/>
-    <col width="45" customWidth="1" min="17" max="17"/>
-    <col width="34" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="17" max="17"/>
+    <col width="55" customWidth="1" min="18" max="18"/>
+    <col width="45" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,50 +557,60 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>The question she's asking</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Hook (answers it, on the pin under the overlay)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Pin title</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Pin description</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Alt text</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Pinterest board</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Amazon affiliate link</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Image prompt (OpenArt / Runway)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Video plan (8-10 sec)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Avatar line (caption or voice)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>File name</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>ASIN</t>
         </is>
@@ -644,50 +658,60 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
+          <t>What do you get a baseball dad who already has everything?</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>The gift he'll use every bullpen: a radar that clocks every pitch.</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
           <t>Baseball Dad Gifts: Pocket Radar Smart Coach</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Baseball dad gifts: the Pocket Radar Smart Coach is a pocket-size radar that reads pitch speed and exit velo, with an app that saves every rep. A smart pick if you're also searching softball dad gifts or baseball coach christmas gifts. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>Dad behind a backstop at dusk holding a small black device, teen pitcher blurred in background, with the words "baseball dad gifts" across the top.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Sports Dad Essentials &amp; Gifts</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B07H7SN831?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, dad behind a backstop at dusk holding a small black device, teen pitcher blurred in background. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "baseball dad gifts". Shot 2 (5s): dad behind a backstop at dusk holding a small black device, teen pitcher blurred in background. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>Searching baseball dad gifts? Here's one parents are buying: the Pocket Radar Smart Coach. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>day001-01-baseball-dad-gifts</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>B07H7SN831</t>
         </is>
@@ -735,50 +759,60 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
+          <t>What Christmas gift will a teen athlete actually use?</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>The recovery tool they'll grab after every practice.</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
           <t>Christmas Gifts for Teen Athletes: Theragun Relief</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Christmas gifts for teen athletes: the Theragun Relief is a lightweight massage gun for sore legs after practice and long tournament weekends. A smart pick if you're also searching christmas gifts athletes or gifts for athletes. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Wrapped gift box under a Christmas tree next to a teen's cleats and gym bag, with the words "christmas gifts for teen athletes" across the top.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>Sports Mom Gifts &amp; Gift Baskets</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0CNS894RH?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, wrapped gift box under a Christmas tree next to a teen's cleats and gym bag. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "christmas gifts for teen athletes". Shot 2 (5s): wrapped gift box under a Christmas tree next to a teen's cleats and gym bag. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="S3" s="4" t="inlineStr">
         <is>
           <t>Searching christmas gifts for teen athletes? Here's one parents are buying: the Theragun Relief. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>day001-02-christmas-gifts-for-teen-athletes</t>
         </is>
       </c>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="U3" s="2" t="inlineStr">
         <is>
           <t>B0CNS894RH</t>
         </is>
@@ -826,50 +860,60 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
+          <t>Which backyard hoop grows with my kid?</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>The height adjusts as they grow, so you only buy one hoop.</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
           <t>Backyard Basketball Hoop: Lifetime portable hoop</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Backyard basketball hoop: the Lifetime portable hoop is an adjustable-height portable hoop that grows with your player from driveway games to real reps. A smart pick if you're also searching backyard basketball court ideas or basketball christmas gifts ideas. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Suburban driveway at golden hour, portable basketball hoop, kid shooting a jump shot, no logos, with the words "backyard basketball hoop" across the top.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Backyard Sports Training Equipment</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0FS8T1WQW?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, suburban driveway at golden hour, portable basketball hoop, kid shooting a jump shot, no logos. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P4" s="4" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "backyard basketball hoop". Shot 2 (5s): suburban driveway at golden hour, portable basketball hoop, kid shooting a jump shot, no logos. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q4" s="4" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>Searching backyard basketball hoop? Here's one parents are buying: the Lifetime portable hoop. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>day001-03-backyard-basketball-hoop</t>
         </is>
       </c>
-      <c r="S4" s="2" t="inlineStr">
+      <c r="U4" s="2" t="inlineStr">
         <is>
           <t>B0FS8T1WQW</t>
         </is>
@@ -917,50 +961,60 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
+          <t>How do I film my kid's games without shaky video?</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Clip in your phone and it follows the play for you.</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
           <t>Sports Filming: DJI Osmo Mobile 8</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Sports filming: the DJI Osmo Mobile 8 is a phone gimbal that tracks your kid down the field and keeps the video smooth, plus a clip-on mic. A smart pick if you're also searching sports camera shots or christmas gifts for sports mom. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Mom in the bleachers filming a youth soccer game on a phone mounted on a small gimbal, with the words "sports filming" across the top.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>Sports Mom Gifts &amp; Gift Baskets</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0GR9YG1LY?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, mom in the bleachers filming a youth soccer game on a phone mounted on a small gimbal. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="R5" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "sports filming". Shot 2 (5s): mom in the bleachers filming a youth soccer game on a phone mounted on a small gimbal. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
+      <c r="S5" s="4" t="inlineStr">
         <is>
           <t>Searching sports filming? Here's one parents are buying: the DJI Osmo Mobile 8. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>day001-04-sports-filming</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr">
+      <c r="U5" s="2" t="inlineStr">
         <is>
           <t>B0GR9YG1LY</t>
         </is>
@@ -1008,50 +1062,60 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
+          <t>What do you get a runner who has everything?</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>A GPS watch that tracks every mile, split and pace.</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
           <t>Christmas Gifts for Track Runners: Garmin Forerunner 165</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Christmas gifts for track runners: the Garmin Forerunner 165 is a GPS running watch that tracks pace, distance and training load for cross country and track kids. A smart pick if you're also searching gifts for girls in track or track gifts ideas. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Close-up of a runner's wrist at a high school track at sunrise, generic black sports watch, with the words "christmas gifts for track runners" across the top.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>Sports Mom Gifts &amp; Gift Baskets</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0CT3SGHXL?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, close-up of a runner's wrist at a high school track at sunrise, generic black sports watch. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "christmas gifts for track runners". Shot 2 (5s): close-up of a runner's wrist at a high school track at sunrise, generic black sports watch. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
+      <c r="S6" s="4" t="inlineStr">
         <is>
           <t>Searching christmas gifts for track runners? Here's one parents are buying: the Garmin Forerunner 165. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>day001-05-christmas-gifts-for-track-runners</t>
         </is>
       </c>
-      <c r="S6" s="2" t="inlineStr">
+      <c r="U6" s="2" t="inlineStr">
         <is>
           <t>B0CT3SGHXL</t>
         </is>
@@ -1099,50 +1163,60 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
+          <t>How do I survive 3 hours on metal bleachers?</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Back support plus two heat zones. Your back will thank you.</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
           <t>Stadium Seats for Bleachers: heated stadium seat</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Stadium seats for bleachers: the heated stadium seat is a padded bleacher seat with back support and two heat zones, powered by a battery pack. A smart pick if you're also searching cold football games or sports mom cold weather essentials. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Navy padded stadium seat on metal bleachers under Friday night lights, breath visible in cold air, with the words "stadium seats for bleachers" across the top.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>Stadium Seats &amp; Bleacher Comfort</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="P7" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0C2YCMB3R?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, navy padded stadium seat on metal bleachers under Friday night lights, breath visible in cold air. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P7" s="4" t="inlineStr">
+      <c r="R7" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "stadium seats for bleachers". Shot 2 (5s): navy padded stadium seat on metal bleachers under Friday night lights, breath visible in cold air. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q7" s="4" t="inlineStr">
+      <c r="S7" s="4" t="inlineStr">
         <is>
           <t>Searching stadium seats for bleachers? Here's one parents are buying: the heated stadium seat. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t>day001-06-stadium-seats-for-bleachers</t>
         </is>
       </c>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="U7" s="2" t="inlineStr">
         <is>
           <t>B0C2YCMB3R</t>
         </is>
@@ -1190,50 +1264,60 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
+          <t>How do I stay warm at night games without 5 bulky layers?</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>One thin battery-heated vest under your jacket. That's it.</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
           <t>Sports Mom Cold Weather Essentials: ORORO heated vest</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>Sports mom cold weather essentials: the ORORO heated vest is a lightweight battery-heated vest that layers under a jacket for cold games and early tournaments. A smart pick if you're also searching cold football game fits or winter sports mom essentials. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>Mom in a quilted vest and beanie on bleachers at a night football game, warm stadium lights, with the words "sports mom cold weather essentials" across the top.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>Cold Football Game Essentials</t>
         </is>
       </c>
-      <c r="N8" s="5" t="inlineStr">
+      <c r="P8" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B01H50RF46?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, mom in a quilted vest and beanie on bleachers at a night football game, warm stadium lights. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P8" s="4" t="inlineStr">
+      <c r="R8" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "sports mom cold weather essentials". Shot 2 (5s): mom in a quilted vest and beanie on bleachers at a night football game, warm stadium lights. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr">
+      <c r="S8" s="4" t="inlineStr">
         <is>
           <t>Searching sports mom cold weather essentials? Here's one parents are buying: the ORORO heated vest. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R8" s="2" t="inlineStr">
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>day001-07-sports-mom-cold-weather-essentials</t>
         </is>
       </c>
-      <c r="S8" s="2" t="inlineStr">
+      <c r="U8" s="2" t="inlineStr">
         <is>
           <t>B01H50RF46</t>
         </is>
@@ -1281,50 +1365,60 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
+          <t>What do I get the mom who lives in the bleachers?</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Cozy boots she can slip on before every cold game.</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
           <t>Christmas Gifts for Sports Mom: UGG Ultra Mini</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>Christmas gifts for sports mom: the UGG Ultra Mini is the cozy ankle-height boot that keeps her feet warm on cold bleachers and slips on in seconds. A smart pick if you're also searching sports mom christmas gift or gifts for the sports mom. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Chestnut suede ankle boots on a cozy blanket next to a stadium cup and team scarf, gift-wrap ribbon, with the words "christmas gifts for sports mom" across the top.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>Sports Mom Gifts &amp; Gift Baskets</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="P9" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B082HHTKB6?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="Q9" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, chestnut suede ankle boots on a cozy blanket next to a stadium cup and team scarf, gift-wrap ribbon. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P9" s="4" t="inlineStr">
+      <c r="R9" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "christmas gifts for sports mom". Shot 2 (5s): chestnut suede ankle boots on a cozy blanket next to a stadium cup and team scarf, gift-wrap ribbon. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q9" s="4" t="inlineStr">
+      <c r="S9" s="4" t="inlineStr">
         <is>
           <t>Searching christmas gifts for sports mom? Here's one parents are buying: the UGG Ultra Mini. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R9" s="2" t="inlineStr">
+      <c r="T9" s="2" t="inlineStr">
         <is>
           <t>day001-08-christmas-gifts-for-sports-mom</t>
         </is>
       </c>
-      <c r="S9" s="2" t="inlineStr">
+      <c r="U9" s="2" t="inlineStr">
         <is>
           <t>B082HHTKB6</t>
         </is>
@@ -1372,50 +1466,60 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
+          <t>How do I feed the whole team at a tailgate?</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>One portable griddle: pancakes at 7, burgers at noon.</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
           <t>Tailgate Setup Ideas: Blackstone 22" griddle</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>Tailgate setup ideas: the Blackstone 22" griddle is a portable propane griddle with a hood that cooks breakfast or burgers for the whole team at a tailgate. A smart pick if you're also searching tailgate food ideas or sports dad gifts. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>Tailgate tent at a youth football field, tabletop griddle sizzling pancakes and bacon, families in team colors, with the words "tailgate setup ideas" across the top.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>Sports Dad Essentials &amp; Gifts</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="P10" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B07ZS5RQZ4?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="Q10" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, tailgate tent at a youth football field, tabletop griddle sizzling pancakes and bacon, families in team colors. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P10" s="4" t="inlineStr">
+      <c r="R10" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "tailgate setup ideas". Shot 2 (5s): tailgate tent at a youth football field, tabletop griddle sizzling pancakes and bacon, families in team colors. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="inlineStr">
+      <c r="S10" s="4" t="inlineStr">
         <is>
           <t>Searching tailgate setup ideas? Here's one parents are buying: the Blackstone 22" griddle. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R10" s="2" t="inlineStr">
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t>day001-09-tailgate-setup-ideas</t>
         </is>
       </c>
-      <c r="S10" s="2" t="inlineStr">
+      <c r="U10" s="2" t="inlineStr">
         <is>
           <t>B07ZS5RQZ4</t>
         </is>
@@ -1463,50 +1567,60 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
+          <t>How do I keep phones and fans charged all tournament weekend?</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>A quiet power station that charges everything from your canopy.</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
           <t>Travel Ball Must Haves: Jackery Explorer 300</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>Travel ball must haves: the Jackery Explorer 300 is a quiet battery power station that charges phones, fans, heated seats and a tablet all tournament long. A smart pick if you're also searching travel ball essentials or tournament day essentials. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>Tournament canopy at a baseball complex, compact orange power station charging phones and a fan, wagon nearby, with the words "travel ball must haves" across the top.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>Travel Ball &amp; Tournament Must Haves</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="P11" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B082TMBYR6?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
+      <c r="Q11" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, tournament canopy at a baseball complex, compact orange power station charging phones and a fan, wagon nearby. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P11" s="4" t="inlineStr">
+      <c r="R11" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "travel ball must haves". Shot 2 (5s): tournament canopy at a baseball complex, compact orange power station charging phones and a fan, wagon nearby. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q11" s="4" t="inlineStr">
+      <c r="S11" s="4" t="inlineStr">
         <is>
           <t>Searching travel ball must haves? Here's one parents are buying: the Jackery Explorer 300. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R11" s="2" t="inlineStr">
+      <c r="T11" s="2" t="inlineStr">
         <is>
           <t>day001-10-travel-ball-must-haves</t>
         </is>
       </c>
-      <c r="S11" s="2" t="inlineStr">
+      <c r="U11" s="2" t="inlineStr">
         <is>
           <t>B082TMBYR6</t>
         </is>
@@ -1554,50 +1668,60 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
+          <t>How do we stay warm tailgating before a freezing game?</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>A portable propane heater for the tailgate (check field rules first).</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
           <t>Cold Football Games: Mr. Heater Big Buddy</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>Cold football games: the Mr. Heater Big Buddy is a portable propane heater for tailgates and open-air sidelines (check your field's rules first). A smart pick if you're also searching tailgate ideas or winter sports mom essentials. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>Family tailgate at dusk in winter coats around a red portable heater, steam from hot cocoa cups, with the words "cold football games" across the top.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>Cold Football Game Essentials</t>
         </is>
       </c>
-      <c r="N12" s="5" t="inlineStr">
+      <c r="P12" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B07Q82MG8S?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="Q12" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, family tailgate at dusk in winter coats around a red portable heater, steam from hot cocoa cups. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P12" s="4" t="inlineStr">
+      <c r="R12" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "cold football games". Shot 2 (5s): family tailgate at dusk in winter coats around a red portable heater, steam from hot cocoa cups. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
+      <c r="S12" s="4" t="inlineStr">
         <is>
           <t>Searching cold football games? Here's one parents are buying: the Mr. Heater Big Buddy. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R12" s="2" t="inlineStr">
+      <c r="T12" s="2" t="inlineStr">
         <is>
           <t>day001-11-cold-football-games</t>
         </is>
       </c>
-      <c r="S12" s="2" t="inlineStr">
+      <c r="U12" s="2" t="inlineStr">
         <is>
           <t>B07Q82MG8S</t>
         </is>
@@ -1645,50 +1769,60 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
+          <t>How do I get chairs, cooler and gear to the field in one trip?</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>A double-decker wagon: chairs on top, cooler below, one trip.</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
           <t>Sports Wagon Ideas: double decker sports wagon</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>Sports wagon ideas: the double decker sports wagon is a big folding wagon with a second shelf and brakes, so chairs, coolers and gear make it to the field in one trip. A smart pick if you're also searching sports wagon organization or sports mom wagon. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Loaded double decker wagon rolling across a soccer complex parking lot, chairs and cooler on top, morning light, with the words "sports wagon ideas" across the top.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>Sports Wagon Ideas &amp; Accessories</t>
         </is>
       </c>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="P13" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0G23XKMJL?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
+      <c r="Q13" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, loaded double decker wagon rolling across a soccer complex parking lot, chairs and cooler on top, morning light. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P13" s="4" t="inlineStr">
+      <c r="R13" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "sports wagon ideas". Shot 2 (5s): loaded double decker wagon rolling across a soccer complex parking lot, chairs and cooler on top, morning light. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q13" s="4" t="inlineStr">
+      <c r="S13" s="4" t="inlineStr">
         <is>
           <t>Searching sports wagon ideas? Here's one parents are buying: the double decker sports wagon. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R13" s="2" t="inlineStr">
+      <c r="T13" s="2" t="inlineStr">
         <is>
           <t>day001-12-sports-wagon-ideas</t>
         </is>
       </c>
-      <c r="S13" s="2" t="inlineStr">
+      <c r="U13" s="2" t="inlineStr">
         <is>
           <t>B0G23XKMJL</t>
         </is>
@@ -1736,50 +1870,60 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
+          <t>Where can my gymnast practice tumbling at home?</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>An air track for cartwheels in the living room. Rolls up after.</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
           <t>Gymnastics Gifts for Kids: air track tumbling mat</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>Gymnastics gifts for kids: the air track tumbling mat is an inflatable tumbling track for cartwheels and back walkovers at home, rolls up when practice is over. A smart pick if you're also searching tumbling mats for kids or gymnastics equipment for home. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Living room with a long inflatable tumbling mat, girl mid-cartwheel, holiday decorations in background, with the words "gymnastics gifts for kids" across the top.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>Backyard Sports Training Equipment</t>
         </is>
       </c>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="P14" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B078815CXR?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, living room with a long inflatable tumbling mat, girl mid-cartwheel, holiday decorations in background. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="R14" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "gymnastics gifts for kids". Shot 2 (5s): living room with a long inflatable tumbling mat, girl mid-cartwheel, holiday decorations in background. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="S14" s="4" t="inlineStr">
         <is>
           <t>Searching gymnastics gifts for kids? Here's one parents are buying: the air track tumbling mat. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R14" s="2" t="inlineStr">
+      <c r="T14" s="2" t="inlineStr">
         <is>
           <t>day001-13-gymnastics-gifts-for-kids</t>
         </is>
       </c>
-      <c r="S14" s="2" t="inlineStr">
+      <c r="U14" s="2" t="inlineStr">
         <is>
           <t>B078815CXR</t>
         </is>
@@ -1827,50 +1971,60 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
+          <t>What basketball gift keeps them off screens all winter?</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Two hoops, a scoreboard, and nonstop shooting in the basement.</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
           <t>Basketball Christmas Gifts Ideas: Pop-A-Shot Dual Shot</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>Basketball christmas gifts ideas: the Pop-A-Shot Dual Shot is a two-hoop electronic arcade basketball game for the basement or garage, built for nonstop shooting. A smart pick if you're also searching basketball gifts for boys or sports room for boys. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>Basement game room, two-hoop arcade basketball machine glowing, two siblings shooting, Christmas lights, with the words "basketball christmas gifts ideas" across the top.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>Sports Mom Gifts &amp; Gift Baskets</t>
         </is>
       </c>
-      <c r="N15" s="5" t="inlineStr">
+      <c r="P15" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B07XFPSZ58?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr">
+      <c r="Q15" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, basement game room, two-hoop arcade basketball machine glowing, two siblings shooting, Christmas lights. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P15" s="4" t="inlineStr">
+      <c r="R15" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "basketball christmas gifts ideas". Shot 2 (5s): basement game room, two-hoop arcade basketball machine glowing, two siblings shooting, Christmas lights. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q15" s="4" t="inlineStr">
+      <c r="S15" s="4" t="inlineStr">
         <is>
           <t>Searching basketball christmas gifts ideas? Here's one parents are buying: the Pop-A-Shot Dual Shot. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R15" s="2" t="inlineStr">
+      <c r="T15" s="2" t="inlineStr">
         <is>
           <t>day001-14-basketball-christmas-gifts-ideas</t>
         </is>
       </c>
-      <c r="S15" s="2" t="inlineStr">
+      <c r="U15" s="2" t="inlineStr">
         <is>
           <t>B07XFPSZ58</t>
         </is>
@@ -1918,50 +2072,60 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
+          <t>How do I set up a teen home gym in a small space?</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>One pair of adjustable dumbbells replaces a whole rack.</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
           <t>Home Gym for Teen Boy: BowFlex SelectTech dumbbells</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>Home gym for teen boy: the BowFlex SelectTech dumbbells is adjustable dumbbells that replace a full rack, so a teen athlete can lift at home in a small corner. A smart pick if you're also searching teen home gym ideas or garage gym ideas. Tap to see it on Amazon. Affiliate link: I may earn a small commission at no extra cost to you.</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>Clean garage gym corner with a bench and adjustable dumbbells, teen athlete doing curls, morning light, with the words "home gym for teen boy" across the top.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>Backyard Sports Training Equipment</t>
         </is>
       </c>
-      <c r="N16" s="5" t="inlineStr">
+      <c r="P16" s="5" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0FRNG2N5H?tag=screenfreet0f-20</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
+      <c r="Q16" s="4" t="inlineStr">
         <is>
           <t>Vertical 2:3 photo, clean garage gym corner with a bench and adjustable dumbbells, teen athlete doing curls, morning light. Natural light, candid, realistic. No brand logos, no readable text. Leave the top third clear for a text overlay.</t>
         </is>
       </c>
-      <c r="P16" s="4" t="inlineStr">
+      <c r="R16" s="4" t="inlineStr">
         <is>
           <t>9:16 or 2:3, 8-10 seconds. Shot 1 (3s): your brand avatar at the field/bleachers, looks at camera and points up to the overlay "home gym for teen boy". Shot 2 (5s): clean garage gym corner with a bench and adjustable dumbbells, teen athlete doing curls, morning light. Slow push-in. End card: product name + "Tap the pin".</t>
         </is>
       </c>
-      <c r="Q16" s="4" t="inlineStr">
+      <c r="S16" s="4" t="inlineStr">
         <is>
           <t>Searching home gym for teen boy? Here's one parents are buying: the BowFlex SelectTech dumbbells. Tap the pin to see it.</t>
         </is>
       </c>
-      <c r="R16" s="2" t="inlineStr">
+      <c r="T16" s="2" t="inlineStr">
         <is>
           <t>day001-15-home-gym-for-teen-boy</t>
         </is>
       </c>
-      <c r="S16" s="2" t="inlineStr">
+      <c r="U16" s="2" t="inlineStr">
         <is>
           <t>B0FRNG2N5H</t>
         </is>
@@ -1969,21 +2133,21 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -1998,7 +2162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -2021,35 +2185,42 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>3. No prices, star ratings or review counts on the pin or in the voiceover (Amazon only allows those when pulled live from Amazon).</t>
+          <t>3. Every pin names the question she has when she types that phrase, and the hook (one line under the overlay) answers it. Keep hooks under 75 characters.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>4. No Amazon product photos. Use your own photos, brand-approved media, or AI lifestyle scenes like the prompts here.</t>
+          <t>4. No prices, star ratings or review counts on the pin or in the voiceover (Amazon only allows those when pulled live from Amazon).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>5. Your avatar is a host, not a customer: it can point, explain and say 'parents are buying'. It never says 'I bought/use/love this'.</t>
+          <t>5. No Amazon product photos. Use your own photos, brand-approved media, or AI lifestyle scenes like the prompts here.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>6. Add a small 'AI-generated' note on any pin that uses your AI avatar.</t>
+          <t>6. Your avatar is a host, not a customer: it can point, explain and say 'parents are buying'. It never says 'I bought/use/love this'.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>7. Link straight to Amazon with your tag (screenfreet0f-20). Prices were checked Oct 30; re-check before you post.</t>
+          <t>7. Add a small 'AI-generated' note on any pin that uses your AI avatar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>8. Link straight to Amazon with your tag (screenfreet0f-20). Prices were checked Oct 30; re-check before you post.</t>
         </is>
       </c>
     </row>

</xml_diff>